<commit_message>
sync(workvault): 2026-10-14 14:14 差分 7 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/PanaCIM管理手順書_草案.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/PanaCIM管理手順書_草案.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>0.11(草案・未検証)</t>
+          <t>0.12(草案・未検証)</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -889,7 +889,7 @@
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>出典は 不具合別ログリスト_取得手順_Ｊ.pdf(PDF通し11〜12頁)。原文は付録A-1。</t>
+          <t>2026-10-14 会議で確認された現状: DGS 側でバックアップを実施中。実行は端末ごとの手作業であり、実施時間は端末によってまちまち。Pana-CIM 側で一括・自動化できないかを調査中(第14章 No.11)。</t>
         </is>
       </c>
       <c r="B10" s="15" t="n"/>
@@ -900,97 +900,97 @@
       <c r="G10" s="16" t="n"/>
     </row>
     <row r="11"/>
-    <row r="12" ht="17.5" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>手順1</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>PanaCIM コンソールを起動する</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="17.5" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>手順2</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>「データベースユーティリティ」→「バックアップ」→「バックアップ設定」→「バックアップ実行」のタブを選択する</t>
-        </is>
-      </c>
-    </row>
+    <row r="12" ht="16.5" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>出典は 不具合別ログリスト_取得手順_Ｊ.pdf(PDF通し11〜12頁)。原文は付録A-1。</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="16" t="n"/>
+    </row>
+    <row r="13"/>
     <row r="14" ht="17.5" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>手順3</t>
+          <t>手順1</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>「データベースバックアップ場所」を確認する(例 E:\BackUP_DB)。確認後、「実行開始」をクリックする</t>
+          <t>PanaCIM コンソールを起動する</t>
         </is>
       </c>
     </row>
     <row r="15" ht="17.5" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>手順4</t>
+          <t>手順2</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>保存が完了すると「データベース完全バックアップに成功しました。」が表示される</t>
+          <t>「データベースユーティリティ」→「バックアップ」→「バックアップ設定」→「バックアップ実行」のタブを選択する</t>
         </is>
       </c>
     </row>
     <row r="16" ht="17.5" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>手順5</t>
+          <t>手順3</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>バックアップの場所(例 E:\BackUP_DB)を開く</t>
+          <t>「データベースバックアップ場所」を確認する(例 E:\BackUP_DB)。確認後、「実行開始」をクリックする</t>
         </is>
       </c>
     </row>
     <row r="17" ht="17.5" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
+          <t>手順4</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>保存が完了すると「データベース完全バックアップに成功しました。」が表示される</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="17.5" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>手順5</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>バックアップの場所(例 E:\BackUP_DB)を開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17.5" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
           <t>手順6</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>画面下に PANACIM_&lt;日付&gt;_&lt;時刻&gt;_FULbak のファイルがある。USB や SD カードへコピーする。ファイルサイズが大きいため、コピー後に圧縮する</t>
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19" ht="17.5" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+    <row r="20"/>
+    <row r="21" ht="17.5" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>保存先の表記について。原文のPDFから抽出した文字列は E\BackUP_DB で、ドライブ文字の後のコロンが落ちている。本書では E:\BackUP_DB と書いた。実機の画面で正しい保存先を確認すること(第14章 No.11)。</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="16" t="n"/>
-    </row>
-    <row r="20"/>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>8-2 確定していないこと</t>
         </is>
       </c>
       <c r="B21" s="15" t="n"/>
@@ -1001,100 +1001,115 @@
       <c r="G21" s="16" t="n"/>
     </row>
     <row r="22"/>
-    <row r="23" ht="17.5" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>8-2 確定していないこと</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="16" t="n"/>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="17.5" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>状態</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="17.5" customHeight="1">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ファイル名の正式な命名規則</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>要確認。原文の ****.**.** は抽出時の伏字</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="17.5" customHeight="1">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>外部媒体の種類と管理</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>要確認</t>
         </is>
       </c>
     </row>
     <row r="26" ht="17.5" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
-          <t>保持する世代数と期間</t>
+          <t>ファイル名の正式な命名規則</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>要確認。原文の ****.**.** は抽出時の伏字</t>
         </is>
       </c>
     </row>
     <row r="27" ht="17.5" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
+          <t>外部媒体の種類と管理</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="17.5" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>保持する世代数と期間</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="17.5" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>取得者と取得時刻</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>要確認</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="31" customHeight="1">
-      <c r="A28" t="inlineStr">
+    <row r="30" ht="31" customHeight="1">
+      <c r="A30" t="inlineStr">
         <is>
           <t>成否を確認する担当者</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>要確認。本節で最も重要。現状: L1/L2/L3 それぞれで取得していることは会議で確認済みだが、誰が・いつ・どこに保存しているかは未確認。確認先の候補挙げは篠原が実施し(会議記録 §10 持ち帰りタスク)、実施者の確定は本会議(10-14)で判断する</t>
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30" ht="17.5" customHeight="1">
-      <c r="A30" s="21" t="inlineStr">
+    <row r="31"/>
+    <row r="32" ht="17.5" customHeight="1">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>バックアップ障害は「成否を確認する担当が決まっていなかった」ことで長期化している。Eg-Pro のサブサーバー同期は1年以上、nksv523 は6月から暫定運用のまま。手順書を作るだけでは同じことが起きる。誰がどこで結果を確認し、失敗時に何をするかまで決める。</t>
         </is>
       </c>
-      <c r="B30" s="15" t="n"/>
-      <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="n"/>
-      <c r="G30" s="16" t="n"/>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="16" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId1"/>
@@ -5163,7 +5178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5550,6 +5565,33 @@
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>未</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="31" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>第2回会議(10-14 13:10)の結果を反映。§8 にバックアップの現状（DGS側で実施中・端末ごとの手作業・実施時間はまちまち・Pana-CIM 側一括化を調査中）を追記</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>篠原</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>未</t>
         </is>

</xml_diff>